<commit_message>
feat(import): mejorar gestión de módulos y formatos DIAN en la importación de clientes
- Se actualiza la lógica de importación para que, al dejar en blanco los bloques de módulos y formatos DIAN, se activen todos por defecto. Un "No" explícito ahora excluye módulos y formatos en lugar de activarlos.
- Se añaden nuevas propiedades `modulosEnBlanco` y `dianEnBlanco` al modelo de cliente para reflejar el estado de los bloques durante la importación.
- Se ajustan las pruebas para verificar el comportamiento correcto de la importación con bloques en blanco y con selecciones explícitas.

Verificado: funcionalidad de importación de clientes confirmada, pruebas unitarias actualizadas.
</commit_message>
<xml_diff>
--- a/Plantilla_Importacion_Clientes.xlsx
+++ b/Plantilla_Importacion_Clientes.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="99">
   <si>
     <t xml:space="preserve">Plantilla de importación masiva de clientes</t>
   </si>
@@ -45,7 +45,10 @@
     <t xml:space="preserve">4.  «Tipo de cliente» es A, B o C (lista desplegable).</t>
   </si>
   <si>
-    <t xml:space="preserve">5.  ERP, Sector, Socio, Gerente y Senior tienen lista desplegable. Para módulos y DIAN elige «Sí» o «No» (vacío = No).</t>
+    <t xml:space="preserve">5.  ERP, Sector, Socio, Gerente y Senior tienen lista desplegable.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5b. Módulos y DIAN: déjalos EN BLANCO para activar TODOS por defecto. Marca «Sí»/«No» solo si quieres elegir cuáles.</t>
   </si>
   <si>
     <t xml:space="preserve">6.  «Staff (ejecuta)» admite uno o varios: escribe los nombres separados por punto y coma «;».</t>
@@ -132,7 +135,7 @@
     <t xml:space="preserve">Módulos (6 columnas)</t>
   </si>
   <si>
-    <t xml:space="preserve">Activos fijos, Cartera, Cuentas por pagar, Ingresos, Inventarios, Nómina. Sí/No.</t>
+    <t xml:space="preserve">Activos fijos, Cartera, Cuentas por pagar, Ingresos, Inventarios, Nómina. En blanco = TODOS; «Sí» activa, «No» excluye.</t>
   </si>
   <si>
     <t xml:space="preserve">No</t>
@@ -141,7 +144,7 @@
     <t xml:space="preserve">DIAN (3 columnas)</t>
   </si>
   <si>
-    <t xml:space="preserve">IVA (F-300), Retención en la fuente (F-350), ICA (F-CHIP). Sí/No.</t>
+    <t xml:space="preserve">IVA (F-300), Retención en la fuente (F-350), ICA (F-CHIP). En blanco = TODOS; «Sí» activa, «No» excluye.</t>
   </si>
   <si>
     <t xml:space="preserve">Socios disponibles (firma · informativo)</t>
@@ -881,7 +884,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="B2:E35"/>
+  <dimension ref="B2:E36"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="3"/>
@@ -987,208 +990,216 @@
       <c r="D14" s="4"/>
       <c r="E14" s="4"/>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B16" s="3" t="s">
+    <row r="15" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B15" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="C16" s="3"/>
-      <c r="D16" s="3"/>
-      <c r="E16" s="3"/>
-    </row>
-    <row r="17" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B17" s="5" t="s">
+      <c r="C15" s="4"/>
+      <c r="D15" s="4"/>
+      <c r="E15" s="4"/>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B17" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="C17" s="6" t="s">
+      <c r="C17" s="3"/>
+      <c r="D17" s="3"/>
+      <c r="E17" s="3"/>
+    </row>
+    <row r="18" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B18" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="D17" s="6"/>
-      <c r="E17" s="5" t="s">
+      <c r="C18" s="6" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="18" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B18" s="7" t="s">
+      <c r="D18" s="6"/>
+      <c r="E18" s="5" t="s">
         <v>16</v>
-      </c>
-      <c r="C18" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="D18" s="8"/>
-      <c r="E18" s="9" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B19" s="7" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C19" s="8" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="D19" s="8"/>
       <c r="E19" s="9" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B20" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="C20" s="8" t="s">
         <v>21</v>
-      </c>
-      <c r="C20" s="8" t="s">
-        <v>22</v>
       </c>
       <c r="D20" s="8"/>
       <c r="E20" s="9" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B21" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="C21" s="8" t="s">
         <v>23</v>
-      </c>
-      <c r="C21" s="8" t="s">
-        <v>24</v>
       </c>
       <c r="D21" s="8"/>
       <c r="E21" s="9" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B22" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="C22" s="8" t="s">
         <v>25</v>
-      </c>
-      <c r="C22" s="8" t="s">
-        <v>26</v>
       </c>
       <c r="D22" s="8"/>
       <c r="E22" s="9" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B23" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="C23" s="8" t="s">
         <v>27</v>
-      </c>
-      <c r="C23" s="8" t="s">
-        <v>28</v>
       </c>
       <c r="D23" s="8"/>
       <c r="E23" s="9" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B24" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="C24" s="8" t="s">
         <v>29</v>
-      </c>
-      <c r="C24" s="8" t="s">
-        <v>30</v>
       </c>
       <c r="D24" s="8"/>
       <c r="E24" s="9" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B25" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="C25" s="8" t="s">
         <v>31</v>
-      </c>
-      <c r="C25" s="8" t="s">
-        <v>32</v>
       </c>
       <c r="D25" s="8"/>
       <c r="E25" s="9" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B26" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="C26" s="8" t="s">
         <v>33</v>
-      </c>
-      <c r="C26" s="8" t="s">
-        <v>34</v>
       </c>
       <c r="D26" s="8"/>
       <c r="E26" s="9" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B27" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="C27" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="C27" s="8" t="s">
-        <v>36</v>
-      </c>
       <c r="D27" s="8"/>
-      <c r="E27" s="10" t="s">
-        <v>37</v>
+      <c r="E27" s="9" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B28" s="7" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C28" s="8" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D28" s="8"/>
       <c r="E28" s="10" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B30" s="3" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B29" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="C29" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="C30" s="3"/>
-      <c r="D30" s="3"/>
-      <c r="E30" s="3"/>
-    </row>
-    <row r="31" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B31" s="4" t="s">
+      <c r="D29" s="8"/>
+      <c r="E29" s="10" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B31" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="C31" s="4"/>
-      <c r="D31" s="4"/>
-      <c r="E31" s="4"/>
-    </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B33" s="3" t="s">
+      <c r="C31" s="3"/>
+      <c r="D31" s="3"/>
+      <c r="E31" s="3"/>
+    </row>
+    <row r="32" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B32" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="C33" s="3"/>
-      <c r="D33" s="3"/>
-      <c r="E33" s="3"/>
-    </row>
-    <row r="34" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B34" s="11" t="s">
-        <v>29</v>
-      </c>
-      <c r="C34" s="11" t="s">
-        <v>31</v>
-      </c>
-      <c r="D34" s="11" t="s">
+      <c r="C32" s="4"/>
+      <c r="D32" s="4"/>
+      <c r="E32" s="4"/>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B34" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="E34" s="11"/>
-    </row>
-    <row r="35" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B35" s="8" t="s">
+      <c r="C34" s="3"/>
+      <c r="D34" s="3"/>
+      <c r="E34" s="3"/>
+    </row>
+    <row r="35" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B35" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="C35" s="11" t="s">
+        <v>32</v>
+      </c>
+      <c r="D35" s="11" t="s">
         <v>44</v>
       </c>
-      <c r="C35" s="8" t="s">
+      <c r="E35" s="11"/>
+    </row>
+    <row r="36" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B36" s="8" t="s">
         <v>45</v>
       </c>
-      <c r="D35" s="8" t="s">
+      <c r="C36" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="E35" s="8"/>
+      <c r="D36" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="E36" s="8"/>
     </row>
   </sheetData>
-  <mergeCells count="30">
+  <mergeCells count="31">
     <mergeCell ref="B2:E2"/>
     <mergeCell ref="B3:E3"/>
     <mergeCell ref="B5:E5"/>
@@ -1201,8 +1212,8 @@
     <mergeCell ref="B12:E12"/>
     <mergeCell ref="B13:E13"/>
     <mergeCell ref="B14:E14"/>
-    <mergeCell ref="B16:E16"/>
-    <mergeCell ref="C17:D17"/>
+    <mergeCell ref="B15:E15"/>
+    <mergeCell ref="B17:E17"/>
     <mergeCell ref="C18:D18"/>
     <mergeCell ref="C19:D19"/>
     <mergeCell ref="C20:D20"/>
@@ -1214,11 +1225,12 @@
     <mergeCell ref="C26:D26"/>
     <mergeCell ref="C27:D27"/>
     <mergeCell ref="C28:D28"/>
-    <mergeCell ref="B30:E30"/>
+    <mergeCell ref="C29:D29"/>
     <mergeCell ref="B31:E31"/>
-    <mergeCell ref="B33:E33"/>
-    <mergeCell ref="D34:E34"/>
+    <mergeCell ref="B32:E32"/>
+    <mergeCell ref="B34:E34"/>
     <mergeCell ref="D35:E35"/>
+    <mergeCell ref="D36:E36"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -1250,176 +1262,176 @@
   <sheetData>
     <row r="1" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="12" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C1" s="12" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D1" s="12" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E1" s="12" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="F1" s="12" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="G1" s="12" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="H1" s="12" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="I1" s="12" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="J1" s="13" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="K1" s="13" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="L1" s="13" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="M1" s="13" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="N1" s="13" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="O1" s="13" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="P1" s="13" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="Q1" s="13" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="R1" s="13" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="14" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B2" s="14" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C2" s="15" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D2" s="14" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="E2" s="14" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="F2" s="14" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G2" s="14" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="H2" s="14" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="I2" s="14" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="J2" s="15" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="K2" s="15" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="L2" s="15" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="M2" s="15" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="N2" s="15" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="O2" s="15" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="P2" s="15" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="Q2" s="15" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="R2" s="15" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="T2" s="16" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="14" t="s">
+        <v>74</v>
+      </c>
+      <c r="B3" s="14" t="s">
+        <v>75</v>
+      </c>
+      <c r="C3" s="15" t="s">
+        <v>76</v>
+      </c>
+      <c r="D3" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="E3" s="14" t="s">
+        <v>78</v>
+      </c>
+      <c r="F3" s="14" t="s">
+        <v>71</v>
+      </c>
+      <c r="G3" s="14" t="s">
+        <v>45</v>
+      </c>
+      <c r="H3" s="14" t="s">
+        <v>46</v>
+      </c>
+      <c r="I3" s="14" t="s">
+        <v>47</v>
+      </c>
+      <c r="J3" s="15" t="s">
+        <v>38</v>
+      </c>
+      <c r="K3" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="L3" s="15" t="s">
+        <v>38</v>
+      </c>
+      <c r="M3" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="N3" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="O3" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="P3" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="Q3" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="R3" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="T3" s="16" t="s">
         <v>73</v>
-      </c>
-      <c r="B3" s="14" t="s">
-        <v>74</v>
-      </c>
-      <c r="C3" s="15" t="s">
-        <v>75</v>
-      </c>
-      <c r="D3" s="14" t="s">
-        <v>76</v>
-      </c>
-      <c r="E3" s="14" t="s">
-        <v>77</v>
-      </c>
-      <c r="F3" s="14" t="s">
-        <v>70</v>
-      </c>
-      <c r="G3" s="14" t="s">
-        <v>44</v>
-      </c>
-      <c r="H3" s="14" t="s">
-        <v>45</v>
-      </c>
-      <c r="I3" s="14" t="s">
-        <v>46</v>
-      </c>
-      <c r="J3" s="15" t="s">
-        <v>37</v>
-      </c>
-      <c r="K3" s="15" t="s">
-        <v>18</v>
-      </c>
-      <c r="L3" s="15" t="s">
-        <v>37</v>
-      </c>
-      <c r="M3" s="15" t="s">
-        <v>18</v>
-      </c>
-      <c r="N3" s="15" t="s">
-        <v>18</v>
-      </c>
-      <c r="O3" s="15" t="s">
-        <v>18</v>
-      </c>
-      <c r="P3" s="15" t="s">
-        <v>18</v>
-      </c>
-      <c r="Q3" s="15" t="s">
-        <v>18</v>
-      </c>
-      <c r="R3" s="15" t="s">
-        <v>18</v>
-      </c>
-      <c r="T3" s="16" t="s">
-        <v>72</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7455,141 +7467,141 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="20" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B1" s="20" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C1" s="20" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D1" s="20" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="E1" s="20" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="F1" s="20" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="G1" s="20" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="H1" s="20" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="I1" s="20" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="J1" s="20" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="21" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B2" s="21" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C2" s="21" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D2" s="21" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E2" s="21" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="F2" s="21" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="G2" s="21" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="H2" s="21" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="I2" s="21" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="J2" s="21" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="21" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B3" s="21" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C3" s="21" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D3" s="21" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="G3" s="21" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="H3" s="21" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="I3" s="21" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="J3" s="21" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="21" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C4" s="21" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="H4" s="21" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I4" s="21" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="J4" s="21" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="21" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C5" s="21" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="H5" s="21" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C6" s="21" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="H6" s="21" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C7" s="21" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="H7" s="21" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C8" s="21" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
     </row>
   </sheetData>

</xml_diff>